<commit_message>
tentando corrigir erro da conferencia nordeste
</commit_message>
<xml_diff>
--- a/planilhas-geradas/resultados-fake-2025-07-07.xlsx
+++ b/planilhas-geradas/resultados-fake-2025-07-07.xlsx
@@ -433,7 +433,7 @@
         <v>Fortaleza Tritões</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="E2">
         <v>31</v>
@@ -456,10 +456,10 @@
         <v>Caruaru Wolves</v>
       </c>
       <c r="D3">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F3" t="str">
         <v>Arruda</v>
@@ -479,7 +479,7 @@
         <v>Santa Maria Soldiers</v>
       </c>
       <c r="D4">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -505,7 +505,7 @@
         <v>6</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F5" t="str">
         <v>Agronômica</v>
@@ -525,10 +525,10 @@
         <v>Tubarões do Cerrado</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="F6" t="str">
         <v>Eurico Gaspar Dutra</v>
@@ -548,10 +548,10 @@
         <v>Cavalaria 2 de Julho</v>
       </c>
       <c r="D7">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E7">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="F7" t="str">
         <v>Vila Olímpica</v>
@@ -571,10 +571,10 @@
         <v>Manaus Cavaliers</v>
       </c>
       <c r="D8">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="E8">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F8" t="str">
         <v>CT do Rondoniense</v>
@@ -594,10 +594,10 @@
         <v>Timbó Rex</v>
       </c>
       <c r="D9">
-        <v>37</v>
+        <v>6</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F9" t="str">
         <v>Croco Stadium</v>
@@ -617,10 +617,10 @@
         <v>Calvary Cavaliers</v>
       </c>
       <c r="D10">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="E10">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="F10" t="str">
         <v>Croco Stadium</v>
@@ -640,10 +640,10 @@
         <v>Rio Preto Weilers</v>
       </c>
       <c r="D11">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F11" t="str">
         <v>Casa do Dragão</v>
@@ -663,10 +663,10 @@
         <v>Corinthians Steamrollers</v>
       </c>
       <c r="D12">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E12">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F12" t="str">
         <v>Arena Jaguatirica</v>
@@ -689,7 +689,7 @@
         <v>10</v>
       </c>
       <c r="E13">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F13" t="str">
         <v>Arena Frigo Arnaldo</v>
@@ -709,10 +709,10 @@
         <v>Vasco Almirantes</v>
       </c>
       <c r="D14">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E14">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F14" t="str">
         <v>Campo do Tupy</v>
@@ -732,10 +732,10 @@
         <v>Flamengo Imperadores</v>
       </c>
       <c r="D15">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="E15">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="F15" t="str">
         <v>Centro Esportivo Universo</v>
@@ -755,10 +755,10 @@
         <v>Spartans FA</v>
       </c>
       <c r="D16">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="E16">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F16" t="str">
         <v>CTE UFMG</v>
@@ -778,10 +778,10 @@
         <v>Juventude FA</v>
       </c>
       <c r="D17">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E17">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F17" t="str">
         <v>Arena Canadá</v>
@@ -801,7 +801,7 @@
         <v>Istepôs FA</v>
       </c>
       <c r="D18">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="E18">
         <v>37</v>
@@ -824,10 +824,10 @@
         <v>Manaus FA</v>
       </c>
       <c r="D19">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E19">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F19" t="str">
         <v>Vila Olímpica de Manaus</v>
@@ -847,10 +847,10 @@
         <v>Fortaleza Tritões</v>
       </c>
       <c r="D20">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E20">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="F20" t="str">
         <v>Arruda</v>
@@ -870,10 +870,10 @@
         <v>João Pessoa Espectros</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="E21">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F21" t="str">
         <v>Unifor</v>
@@ -893,10 +893,10 @@
         <v>Caruaru Wolves</v>
       </c>
       <c r="D22">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="E22">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F22" t="str">
         <v>Municipal de Lauro de Freitas</v>
@@ -916,10 +916,10 @@
         <v>Coritiba Crocodiles</v>
       </c>
       <c r="D23">
+        <v>28</v>
+      </c>
+      <c r="E23">
         <v>14</v>
-      </c>
-      <c r="E23">
-        <v>13</v>
       </c>
       <c r="F23" t="str">
         <v>Croco Stadium</v>
@@ -939,10 +939,10 @@
         <v>Brown Spiders</v>
       </c>
       <c r="D24">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E24">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F24" t="str">
         <v>Complexo Esportivo de Timbó</v>
@@ -962,10 +962,10 @@
         <v>Rondonópolis Hawks</v>
       </c>
       <c r="D25">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E25">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F25" t="str">
         <v>Eurico Gaspar Dutra</v>
@@ -985,10 +985,10 @@
         <v>Cruzeiro FA</v>
       </c>
       <c r="D26">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E26">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F26" t="str">
         <v>CT Touchdown</v>
@@ -1008,10 +1008,10 @@
         <v>Ocelots FA</v>
       </c>
       <c r="D27">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E27">
-        <v>37</v>
+        <v>6</v>
       </c>
       <c r="F27" t="str">
         <v>Oswaldo de Carlos</v>
@@ -1031,7 +1031,7 @@
         <v>Locomotiva FA</v>
       </c>
       <c r="D28">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E28">
         <v>10</v>
@@ -1054,10 +1054,10 @@
         <v>Tritões FA</v>
       </c>
       <c r="D29">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E29">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F29" t="str">
         <v>Louzadão</v>
@@ -1077,10 +1077,10 @@
         <v>Galo FA</v>
       </c>
       <c r="D30">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E30">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F30" t="str">
         <v>João Mendes Athayde</v>
@@ -1100,10 +1100,10 @@
         <v>Moura Lacerda Dragons</v>
       </c>
       <c r="D31">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E31">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="F31" t="str">
         <v>CT Touchdown</v>
@@ -1123,10 +1123,10 @@
         <v>Manaus FA</v>
       </c>
       <c r="D32">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="E32">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F32" t="str">
         <v>Rorizão</v>
@@ -1146,10 +1146,10 @@
         <v>Santa Maria Soldiers</v>
       </c>
       <c r="D33">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E33">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F33" t="str">
         <v>Arena Canadá</v>
@@ -1169,10 +1169,10 @@
         <v>Porto Velho Miners</v>
       </c>
       <c r="D34">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E34">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="F34" t="str">
         <v>Vila Olímpica de Manaus</v>
@@ -1192,10 +1192,10 @@
         <v>Juventude FA</v>
       </c>
       <c r="D35">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E35">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F35" t="str">
         <v>Agronômica</v>
@@ -1215,10 +1215,10 @@
         <v>Brown Spiders</v>
       </c>
       <c r="D36">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E36">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="F36" t="str">
         <v>Croco Stadium</v>
@@ -1238,10 +1238,10 @@
         <v>Timbó Rex</v>
       </c>
       <c r="D37">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="E37">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F37" t="str">
         <v>Croco Stadium</v>
@@ -1261,10 +1261,10 @@
         <v>Recife Mariners</v>
       </c>
       <c r="D38">
+        <v>41</v>
+      </c>
+      <c r="E38">
         <v>34</v>
-      </c>
-      <c r="E38">
-        <v>31</v>
       </c>
       <c r="F38" t="str">
         <v>Municipal de Lauro de Freitas</v>
@@ -1284,10 +1284,10 @@
         <v>Ceará Sabres</v>
       </c>
       <c r="D39">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="E39">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="F39" t="str">
         <v>Lacerdão</v>
@@ -1307,10 +1307,10 @@
         <v>João Pessoa Espectros</v>
       </c>
       <c r="D40">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E40">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F40" t="str">
         <v>Unifor</v>
@@ -1330,10 +1330,10 @@
         <v>Moura Lacerda Dragons</v>
       </c>
       <c r="D41">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E41">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F41" t="str">
         <v>Centro Esportivo Universo</v>
@@ -1353,10 +1353,10 @@
         <v>Ocelots FA</v>
       </c>
       <c r="D42">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E42">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="F42" t="str">
         <v>Louzadão</v>
@@ -1379,7 +1379,7 @@
         <v>34</v>
       </c>
       <c r="E43">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F43" t="str">
         <v>CT Touchdown</v>
@@ -1399,7 +1399,7 @@
         <v>Rio Preto Weilers</v>
       </c>
       <c r="D44">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="E44">
         <v>34</v>
@@ -1422,10 +1422,10 @@
         <v>Vasco Almirantes</v>
       </c>
       <c r="D45">
+        <v>7</v>
+      </c>
+      <c r="E45">
         <v>0</v>
-      </c>
-      <c r="E45">
-        <v>41</v>
       </c>
       <c r="F45" t="str">
         <v>CT Touchdown</v>
@@ -1445,10 +1445,10 @@
         <v>Tritões FA</v>
       </c>
       <c r="D46">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E46">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F46" t="str">
         <v>CTE UFMG</v>
@@ -1468,10 +1468,10 @@
         <v>Calvary Cavaliers</v>
       </c>
       <c r="D47">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="E47">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F47" t="str">
         <v>Estádio Caxias do Sul/RS</v>
@@ -1491,10 +1491,10 @@
         <v>Bravos FA</v>
       </c>
       <c r="D48">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="E48">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="F48" t="str">
         <v>Complexo Esportivo de Timbó</v>
@@ -1517,7 +1517,7 @@
         <v>42</v>
       </c>
       <c r="E49">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F49" t="str">
         <v>Estádio da Colina</v>
@@ -1537,10 +1537,10 @@
         <v>Coritiba Crocodiles</v>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E50">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="F50" t="str">
         <v>Estádio dos Eucaliptos</v>
@@ -1560,10 +1560,10 @@
         <v>Istepôs FA</v>
       </c>
       <c r="D51">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E51">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F51" t="str">
         <v>Croco Stadium</v>
@@ -1583,10 +1583,10 @@
         <v>Galo FA</v>
       </c>
       <c r="D52">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E52">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F52" t="str">
         <v>Casa do Dragão</v>
@@ -1606,10 +1606,10 @@
         <v>Cruzeiro FA</v>
       </c>
       <c r="D53">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E53">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="F53" t="str">
         <v>Arena Jaguatirica</v>
@@ -1632,7 +1632,7 @@
         <v>17</v>
       </c>
       <c r="E54">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="F54" t="str">
         <v>Oswaldo de Carlos</v>
@@ -1652,10 +1652,10 @@
         <v>Ceará Sabres</v>
       </c>
       <c r="D55">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="E55">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F55" t="str">
         <v>Unifor</v>
@@ -1675,10 +1675,10 @@
         <v>Recife Mariners</v>
       </c>
       <c r="D56">
+        <v>38</v>
+      </c>
+      <c r="E56">
         <v>13</v>
-      </c>
-      <c r="E56">
-        <v>16</v>
       </c>
       <c r="F56" t="str">
         <v>Vila Olímpica</v>
@@ -1698,10 +1698,10 @@
         <v>Cavalaria 2 de Julho</v>
       </c>
       <c r="D57">
+        <v>20</v>
+      </c>
+      <c r="E57">
         <v>9</v>
-      </c>
-      <c r="E57">
-        <v>14</v>
       </c>
       <c r="F57" t="str">
         <v>Lacerdão</v>
@@ -1721,10 +1721,10 @@
         <v>Flamengo Imperadores</v>
       </c>
       <c r="D58">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="E58">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="F58" t="str">
         <v>Municipal José Maria Brito de Barros</v>
@@ -1744,10 +1744,10 @@
         <v>Locomotiva FA</v>
       </c>
       <c r="D59">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="E59">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F59" t="str">
         <v>Campo do Tupy</v>
@@ -1767,10 +1767,10 @@
         <v>Spartans FA</v>
       </c>
       <c r="D60">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E60">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F60" t="str">
         <v>João Mendes Athayde</v>
@@ -1790,10 +1790,10 @@
         <v>Cuiabá Arsenal</v>
       </c>
       <c r="D61">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="E61">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="F61" t="str">
         <v>CT do Tigrão</v>
@@ -1813,10 +1813,10 @@
         <v>Tubarões do Cerrado</v>
       </c>
       <c r="D62">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E62">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F62" t="str">
         <v>CT do Tigrão</v>
@@ -1836,10 +1836,10 @@
         <v>Cuiabá Arsenal</v>
       </c>
       <c r="D63">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E63">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="F63" t="str">
         <v>CT do Rondoniense</v>
@@ -1859,10 +1859,10 @@
         <v>Rondonópolis Hawks</v>
       </c>
       <c r="D64">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E64">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="F64" t="str">
         <v>Rorizão</v>
@@ -1882,10 +1882,10 @@
         <v>Porto Velho Miners</v>
       </c>
       <c r="D65">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="E65">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F65" t="str">
         <v>Estádio da Colina</v>

</xml_diff>